<commit_message>
Fix downloadable template wrapping header sizes and full preview background
</commit_message>
<xml_diff>
--- a/assets/report_templates/MSME_Report_Blank.xlsx
+++ b/assets/report_templates/MSME_Report_Blank.xlsx
@@ -918,12 +918,18 @@
     </xf>
   </cellStyleXfs>
   <cellXfs count="51">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -940,7 +946,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -958,7 +964,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -975,28 +981,48 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" wrapText="1" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment wrapText="1" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1007,7 +1033,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1016,7 +1042,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1031,7 +1057,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment wrapText="1" vertical="center"/>
     </xf>
     <xf numFmtId="178" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1329,7 +1355,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="6600000" cy="750000"/>
+    <xdr:ext cx="11430000" cy="1298864"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="PESO Vinzons letterhead"/>
@@ -1552,25 +1578,38 @@
   <dimension ref="A1:AC345"/>
   <sheetFormatPr defaultColWidth="12.6296296296296" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="3" max="3" width="22.5" customWidth="1"/>
-    <col min="4" max="4" width="21.1296296296296" customWidth="1"/>
-    <col min="5" max="5" width="18.75" customWidth="1"/>
-    <col min="6" max="6" width="25.5" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="10" max="10" width="16.3796296296296" customWidth="1"/>
-    <col min="13" max="13" width="13.8796296296296" customWidth="1"/>
-    <col min="14" max="14" width="21" customWidth="1"/>
-    <col min="15" max="15" width="17.25" customWidth="1"/>
-    <col min="19" max="19" width="18.6296296296296" customWidth="1"/>
-    <col min="21" max="21" width="14" customWidth="1"/>
-    <col min="22" max="22" width="30.25" customWidth="1"/>
-    <col min="23" max="23" width="17.6296296296296" customWidth="1"/>
-    <col min="24" max="24" width="21" customWidth="1"/>
-    <col min="27" max="27" width="15.6296296296296" customWidth="1"/>
-    <col min="28" max="28" width="16.75" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="26" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="26" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
+    <col min="8" max="8" width="26" customWidth="1"/>
+    <col min="9" max="9" width="26" customWidth="1"/>
+    <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="11" max="11" width="22" customWidth="1"/>
+    <col min="12" max="12" width="22" customWidth="1"/>
+    <col min="13" max="13" width="22" customWidth="1"/>
+    <col min="14" max="14" width="18" customWidth="1"/>
+    <col min="15" max="15" width="22" customWidth="1"/>
+    <col min="16" max="16" width="26" customWidth="1"/>
+    <col min="17" max="17" width="22" customWidth="1"/>
+    <col min="18" max="18" width="10" customWidth="1"/>
+    <col min="19" max="19" width="20" customWidth="1"/>
+    <col min="20" max="20" width="8" customWidth="1"/>
+    <col min="21" max="21" width="18" customWidth="1"/>
+    <col min="22" max="22" width="34" customWidth="1"/>
+    <col min="23" max="23" width="22" customWidth="1"/>
+    <col min="24" max="24" width="26" customWidth="1"/>
+    <col min="25" max="25" width="22" customWidth="1"/>
+    <col min="26" max="26" width="18" customWidth="1"/>
+    <col min="27" max="27" width="26" customWidth="1"/>
+    <col min="28" max="28" width="22" customWidth="1"/>
+    <col min="29" max="29" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:29" ht="64">
+    <row r="1" customHeight="1" spans="1:29" ht="110">
       <c r="A1" s="31"/>
       <c r="B1" s="31"/>
       <c r="C1" s="31"/>
@@ -1675,7 +1714,7 @@
       <c r="AB3" s="3"/>
       <c r="AC3" s="37"/>
     </row>
-    <row r="4" customHeight="1" spans="1:29">
+    <row r="4" customHeight="1" spans="1:29" ht="72">
       <c r="A4" s="31"/>
       <c r="B4" s="38"/>
       <c r="C4" s="39" t="inlineStr">
@@ -12785,24 +12824,35 @@
   <dimension ref="A5:Z317"/>
   <sheetFormatPr defaultColWidth="12.6296296296296" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="8.5" customWidth="1"/>
-    <col min="5" max="5" width="17.5" customWidth="1"/>
-    <col min="6" max="7" width="19.25" customWidth="1"/>
-    <col min="9" max="9" width="15.25" customWidth="1"/>
-    <col min="10" max="10" width="14.75" customWidth="1"/>
-    <col min="11" max="11" width="15.5" customWidth="1"/>
-    <col min="12" max="12" width="23.75" customWidth="1"/>
-    <col min="13" max="13" width="19.5" customWidth="1"/>
-    <col min="14" max="14" width="15.1296296296296" customWidth="1"/>
-    <col min="15" max="15" width="26.1296296296296" customWidth="1"/>
-    <col min="16" max="16" width="20.6296296296296" customWidth="1"/>
-    <col min="17" max="17" width="43.5" customWidth="1"/>
-    <col min="18" max="18" width="40.75" customWidth="1"/>
-    <col min="19" max="19" width="37.1296296296296" customWidth="1"/>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="30" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="30" customWidth="1"/>
+    <col min="11" max="11" width="30" customWidth="1"/>
+    <col min="12" max="12" width="30" customWidth="1"/>
+    <col min="13" max="13" width="22" customWidth="1"/>
+    <col min="14" max="14" width="22" customWidth="1"/>
+    <col min="15" max="15" width="30" customWidth="1"/>
+    <col min="16" max="16" width="22" customWidth="1"/>
+    <col min="17" max="17" width="22" customWidth="1"/>
+    <col min="18" max="18" width="22" customWidth="1"/>
+    <col min="19" max="19" width="22" customWidth="1"/>
+    <col min="20" max="20" width="18" customWidth="1"/>
+    <col min="21" max="21" width="18" customWidth="1"/>
+    <col min="22" max="22" width="18" customWidth="1"/>
+    <col min="23" max="23" width="18" customWidth="1"/>
+    <col min="24" max="24" width="18" customWidth="1"/>
+    <col min="25" max="25" width="18" customWidth="1"/>
+    <col min="26" max="26" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="64" customHeight="1"/>
+    <row r="1" ht="110" customHeight="1"/>
     <row r="5" ht="14.7" spans="1:26">
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -12842,7 +12892,7 @@
       <c r="U5" s="7"/>
       <c r="V5" s="8"/>
     </row>
-    <row r="6" ht="67.5" spans="1:26">
+    <row r="6" ht="72" spans="1:26" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
           <t>No</t>

</xml_diff>

<commit_message>
Complete import grids and clean original workbook headings and letterheads
</commit_message>
<xml_diff>
--- a/assets/report_templates/MSME_Report_Blank.xlsx
+++ b/assets/report_templates/MSME_Report_Blank.xlsx
@@ -917,7 +917,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="125">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1" vertical="center"/>
     </xf>
@@ -1070,6 +1070,228 @@
     </xf>
     <xf numFmtId="180" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1355,7 +1577,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="11430000" cy="1298864"/>
+    <xdr:ext cx="13906500" cy="1580300"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="PESO Vinzons letterhead"/>
@@ -1609,7 +1831,7 @@
     <col min="29" max="29" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:29" ht="110">
+    <row r="1" customHeight="1" spans="1:29" ht="140">
       <c r="A1" s="31"/>
       <c r="B1" s="31"/>
       <c r="C1" s="31"/>
@@ -1672,182 +1894,182 @@
       <c r="AC2" s="31"/>
     </row>
     <row r="3" customHeight="1" spans="1:29">
-      <c r="A3" s="31"/>
-      <c r="B3" s="32" t="inlineStr">
+      <c r="A3" s="101"/>
+      <c r="B3" s="102" t="inlineStr">
         <is>
           <t>I. BUSINESS PROFILE</t>
         </is>
       </c>
-      <c r="C3" s="33"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33"/>
-      <c r="I3" s="33"/>
-      <c r="J3" s="33"/>
-      <c r="K3" s="33"/>
-      <c r="L3" s="33"/>
-      <c r="M3" s="33"/>
-      <c r="N3" s="33"/>
-      <c r="O3" s="34"/>
-      <c r="P3" s="35" t="inlineStr">
+      <c r="C3" s="103"/>
+      <c r="D3" s="103"/>
+      <c r="E3" s="103"/>
+      <c r="F3" s="103"/>
+      <c r="G3" s="103"/>
+      <c r="H3" s="103"/>
+      <c r="I3" s="103"/>
+      <c r="J3" s="103"/>
+      <c r="K3" s="103"/>
+      <c r="L3" s="103"/>
+      <c r="M3" s="103"/>
+      <c r="N3" s="103"/>
+      <c r="O3" s="104"/>
+      <c r="P3" s="105" t="inlineStr">
         <is>
           <t>II. OWNER/ENTREPRENEUR INFORMATION</t>
         </is>
       </c>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
-      <c r="S3" s="2"/>
-      <c r="T3" s="2"/>
-      <c r="U3" s="2"/>
-      <c r="V3" s="2"/>
-      <c r="W3" s="2"/>
-      <c r="X3" s="3"/>
-      <c r="Y3" s="36" t="inlineStr">
+      <c r="Q3" s="106"/>
+      <c r="R3" s="106"/>
+      <c r="S3" s="106"/>
+      <c r="T3" s="106"/>
+      <c r="U3" s="106"/>
+      <c r="V3" s="106"/>
+      <c r="W3" s="106"/>
+      <c r="X3" s="107"/>
+      <c r="Y3" s="108" t="inlineStr">
         <is>
           <t>III. BUSINESS OPERATIONS</t>
         </is>
       </c>
-      <c r="Z3" s="2"/>
-      <c r="AA3" s="2"/>
-      <c r="AB3" s="3"/>
-      <c r="AC3" s="37"/>
-    </row>
-    <row r="4" customHeight="1" spans="1:29" ht="72">
-      <c r="A4" s="31"/>
-      <c r="B4" s="38"/>
-      <c r="C4" s="39" t="inlineStr">
+      <c r="Z3" s="106"/>
+      <c r="AA3" s="106"/>
+      <c r="AB3" s="107"/>
+      <c r="AC3" s="109"/>
+    </row>
+    <row r="4" customHeight="1" spans="1:29" ht="90">
+      <c r="A4" s="101"/>
+      <c r="B4" s="110"/>
+      <c r="C4" s="111" t="inlineStr">
         <is>
           <t>Business/Trade Name</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D4" s="112" t="inlineStr">
         <is>
           <t>Type of ownership</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="E4" s="112" t="inlineStr">
         <is>
           <t>Nature of Business</t>
         </is>
       </c>
-      <c r="F4" s="10" t="inlineStr">
+      <c r="F4" s="112" t="inlineStr">
         <is>
           <t>Primary Products offered</t>
         </is>
       </c>
-      <c r="G4" s="10" t="inlineStr">
+      <c r="G4" s="112" t="inlineStr">
         <is>
           <t>Product Price</t>
         </is>
       </c>
-      <c r="H4" s="10" t="inlineStr">
+      <c r="H4" s="112" t="inlineStr">
         <is>
           <t>Year Business Started</t>
         </is>
       </c>
-      <c r="I4" s="10" t="inlineStr">
+      <c r="I4" s="112" t="inlineStr">
         <is>
           <t>Business Permit No:</t>
         </is>
       </c>
-      <c r="J4" s="10" t="inlineStr">
+      <c r="J4" s="112" t="inlineStr">
         <is>
           <t>Valid Until</t>
         </is>
       </c>
-      <c r="K4" s="10" t="inlineStr">
+      <c r="K4" s="112" t="inlineStr">
         <is>
           <t>DTI Registration No.</t>
         </is>
       </c>
-      <c r="L4" s="10" t="inlineStr">
+      <c r="L4" s="112" t="inlineStr">
         <is>
           <t>Tax Identification No. (TIN)</t>
         </is>
       </c>
-      <c r="M4" s="10" t="inlineStr">
+      <c r="M4" s="112" t="inlineStr">
         <is>
           <t>Landline/Mobile Number</t>
         </is>
       </c>
-      <c r="N4" s="10" t="inlineStr">
+      <c r="N4" s="112" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="O4" s="10" t="inlineStr">
+      <c r="O4" s="112" t="inlineStr">
         <is>
           <t>Website/Social Media</t>
         </is>
       </c>
-      <c r="P4" s="10" t="inlineStr">
+      <c r="P4" s="112" t="inlineStr">
         <is>
           <t>Full Name</t>
         </is>
       </c>
-      <c r="Q4" s="10" t="inlineStr">
+      <c r="Q4" s="112" t="inlineStr">
         <is>
           <t>Contact Number</t>
         </is>
       </c>
-      <c r="R4" s="40" t="inlineStr">
+      <c r="R4" s="113" t="inlineStr">
         <is>
           <t>Sex</t>
         </is>
       </c>
-      <c r="S4" s="10" t="inlineStr">
+      <c r="S4" s="112" t="inlineStr">
         <is>
           <t>Date of Birth</t>
         </is>
       </c>
-      <c r="T4" s="10" t="inlineStr">
+      <c r="T4" s="112" t="inlineStr">
         <is>
           <t>Age</t>
         </is>
       </c>
-      <c r="U4" s="10" t="inlineStr">
+      <c r="U4" s="112" t="inlineStr">
         <is>
           <t>Civil Status</t>
         </is>
       </c>
-      <c r="V4" s="10" t="inlineStr">
+      <c r="V4" s="112" t="inlineStr">
         <is>
           <t>Complete Address</t>
         </is>
       </c>
-      <c r="W4" s="10" t="inlineStr">
+      <c r="W4" s="112" t="inlineStr">
         <is>
           <t>Educational Attainment</t>
         </is>
       </c>
-      <c r="X4" s="10" t="inlineStr">
+      <c r="X4" s="112" t="inlineStr">
         <is>
           <t>Current Work/Business Experience</t>
         </is>
       </c>
-      <c r="Y4" s="12" t="inlineStr">
+      <c r="Y4" s="114" t="inlineStr">
         <is>
           <t>Night Market Stall/Booth No.</t>
         </is>
       </c>
-      <c r="Z4" s="12" t="inlineStr">
+      <c r="Z4" s="114" t="inlineStr">
         <is>
           <t>Date Started</t>
         </is>
       </c>
-      <c r="AA4" s="13" t="inlineStr">
+      <c r="AA4" s="115" t="inlineStr">
         <is>
           <t>Business Assets Owned</t>
         </is>
       </c>
-      <c r="AB4" s="13" t="inlineStr">
+      <c r="AB4" s="115" t="inlineStr">
         <is>
           <t>Utility Needs </t>
         </is>
       </c>
-      <c r="AC4" s="37"/>
+      <c r="AC4" s="109"/>
     </row>
     <row r="5" customHeight="1" spans="1:29">
       <c r="A5" s="31"/>
@@ -12852,145 +13074,145 @@
     <col min="26" max="26" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="110" customHeight="1"/>
+    <row r="1" ht="140" customHeight="1"/>
     <row r="5" ht="14.7" spans="1:26">
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B5" s="116" t="inlineStr">
         <is>
           <t>IV. HUMAN RESOURCES</t>
         </is>
       </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="C5" s="106"/>
+      <c r="D5" s="106"/>
+      <c r="E5" s="107"/>
+      <c r="F5" s="117" t="inlineStr">
         <is>
           <t>V. FINANCIAL INFORMATION</t>
         </is>
       </c>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="3"/>
-      <c r="N5" s="5" t="inlineStr">
+      <c r="G5" s="106"/>
+      <c r="H5" s="106"/>
+      <c r="I5" s="106"/>
+      <c r="J5" s="106"/>
+      <c r="K5" s="106"/>
+      <c r="L5" s="106"/>
+      <c r="M5" s="107"/>
+      <c r="N5" s="118" t="inlineStr">
         <is>
           <t>VI. GOVERNMENT ASSISTANCE/PROGRAMS AVAILED</t>
         </is>
       </c>
-      <c r="O5" s="2"/>
-      <c r="P5" s="2"/>
-      <c r="Q5" s="3"/>
-      <c r="R5" s="6" t="inlineStr">
+      <c r="O5" s="106"/>
+      <c r="P5" s="106"/>
+      <c r="Q5" s="107"/>
+      <c r="R5" s="119" t="inlineStr">
         <is>
           <t>VII. CHALLENGES ENCOUNTERED IN BUSINESS</t>
         </is>
       </c>
-      <c r="S5" s="3"/>
-      <c r="T5" s="7"/>
-      <c r="U5" s="7"/>
-      <c r="V5" s="8"/>
-    </row>
-    <row r="6" ht="72" spans="1:26" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="S5" s="107"/>
+      <c r="T5" s="120"/>
+      <c r="U5" s="120"/>
+      <c r="V5" s="121"/>
+    </row>
+    <row r="6" ht="90" spans="1:26" customHeight="1">
+      <c r="A6" s="122" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="112" t="inlineStr">
         <is>
           <t>Number of Workers (M&amp;F)</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="123" t="inlineStr">
         <is>
           <t>Employment Status</t>
         </is>
       </c>
-      <c r="D6" s="3"/>
-      <c r="E6" s="10" t="inlineStr">
+      <c r="D6" s="107"/>
+      <c r="E6" s="112" t="inlineStr">
         <is>
           <t>Skills Training Methold</t>
         </is>
       </c>
-      <c r="F6" s="10" t="inlineStr">
+      <c r="F6" s="112" t="inlineStr">
         <is>
           <t>Source of Capital</t>
         </is>
       </c>
-      <c r="G6" s="10" t="inlineStr">
+      <c r="G6" s="112" t="inlineStr">
         <is>
           <t>Business Size (RA 9501 - Magna Carta for MSMEs)</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
+      <c r="H6" s="112" t="inlineStr">
         <is>
           <t>Amount of Initial Capital</t>
         </is>
       </c>
-      <c r="I6" s="10" t="inlineStr">
+      <c r="I6" s="112" t="inlineStr">
         <is>
           <t>Current Estimated Capital</t>
         </is>
       </c>
-      <c r="J6" s="10" t="inlineStr">
+      <c r="J6" s="112" t="inlineStr">
         <is>
           <t>How much does your business earn on regular business days?</t>
         </is>
       </c>
-      <c r="K6" s="10" t="inlineStr">
+      <c r="K6" s="112" t="inlineStr">
         <is>
           <t>How much did you earn for the two days night market every week?</t>
         </is>
       </c>
-      <c r="L6" s="10" t="inlineStr">
+      <c r="L6" s="112" t="inlineStr">
         <is>
           <t>How much have you earned since you started selling at night market?</t>
         </is>
       </c>
-      <c r="M6" s="10" t="inlineStr">
+      <c r="M6" s="112" t="inlineStr">
         <is>
           <t>Mode of Payment Accepted</t>
         </is>
       </c>
-      <c r="N6" s="10" t="inlineStr">
+      <c r="N6" s="112" t="inlineStr">
         <is>
           <t>Distribution Channels</t>
         </is>
       </c>
-      <c r="O6" s="12" t="inlineStr">
+      <c r="O6" s="114" t="inlineStr">
         <is>
           <t>Have you availed any government programs/support?</t>
         </is>
       </c>
-      <c r="P6" s="12" t="inlineStr">
+      <c r="P6" s="114" t="inlineStr">
         <is>
           <t>If Yes, please specify</t>
         </is>
       </c>
-      <c r="Q6" s="12" t="inlineStr">
+      <c r="Q6" s="114" t="inlineStr">
         <is>
           <t>Programs/Services Availed in the Past</t>
         </is>
       </c>
-      <c r="R6" s="13" t="inlineStr">
+      <c r="R6" s="115" t="inlineStr">
         <is>
           <t>Programs/Services Needed</t>
         </is>
       </c>
-      <c r="S6" s="10" t="inlineStr">
+      <c r="S6" s="112" t="inlineStr">
         <is>
           <t>Please sellect what applies</t>
         </is>
       </c>
-      <c r="T6" s="14"/>
-      <c r="U6" s="14"/>
-      <c r="V6" s="14"/>
-      <c r="W6" s="14"/>
-      <c r="X6" s="14"/>
-      <c r="Y6" s="14"/>
-      <c r="Z6" s="14"/>
+      <c r="T6" s="124"/>
+      <c r="U6" s="124"/>
+      <c r="V6" s="124"/>
+      <c r="W6" s="124"/>
+      <c r="X6" s="124"/>
+      <c r="Y6" s="124"/>
+      <c r="Z6" s="124"/>
     </row>
     <row r="7" ht="13.95" spans="1:26">
       <c r="A7" s="15">
@@ -13014,13 +13236,13 @@
       <c r="Q7" s="19"/>
       <c r="R7" s="19"/>
       <c r="S7" s="19"/>
-      <c r="T7" s="14"/>
-      <c r="U7" s="14"/>
-      <c r="V7" s="14"/>
-      <c r="W7" s="14"/>
-      <c r="X7" s="14"/>
-      <c r="Y7" s="14"/>
-      <c r="Z7" s="14"/>
+      <c r="T7" s="99"/>
+      <c r="U7" s="99"/>
+      <c r="V7" s="99"/>
+      <c r="W7" s="99"/>
+      <c r="X7" s="99"/>
+      <c r="Y7" s="99"/>
+      <c r="Z7" s="99"/>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:26">
       <c r="A8" s="21"/>
@@ -13042,13 +13264,13 @@
       <c r="Q8" s="24"/>
       <c r="R8" s="24"/>
       <c r="S8" s="24"/>
-      <c r="T8" s="14"/>
-      <c r="U8" s="14"/>
-      <c r="V8" s="14"/>
-      <c r="W8" s="14"/>
-      <c r="X8" s="14"/>
-      <c r="Y8" s="14"/>
-      <c r="Z8" s="14"/>
+      <c r="T8" s="99"/>
+      <c r="U8" s="99"/>
+      <c r="V8" s="99"/>
+      <c r="W8" s="99"/>
+      <c r="X8" s="99"/>
+      <c r="Y8" s="99"/>
+      <c r="Z8" s="99"/>
     </row>
     <row r="9" ht="13.2" spans="1:26">
       <c r="A9" s="21"/>
@@ -13070,13 +13292,13 @@
       <c r="Q9" s="24"/>
       <c r="R9" s="24"/>
       <c r="S9" s="24"/>
-      <c r="T9" s="14"/>
-      <c r="U9" s="14"/>
-      <c r="V9" s="14"/>
-      <c r="W9" s="14"/>
-      <c r="X9" s="14"/>
-      <c r="Y9" s="14"/>
-      <c r="Z9" s="14"/>
+      <c r="T9" s="99"/>
+      <c r="U9" s="99"/>
+      <c r="V9" s="99"/>
+      <c r="W9" s="99"/>
+      <c r="X9" s="99"/>
+      <c r="Y9" s="99"/>
+      <c r="Z9" s="99"/>
     </row>
     <row r="10" ht="13.2" spans="1:26">
       <c r="A10" s="21"/>
@@ -13098,13 +13320,13 @@
       <c r="Q10" s="24"/>
       <c r="R10" s="24"/>
       <c r="S10" s="24"/>
-      <c r="T10" s="14"/>
-      <c r="U10" s="14"/>
-      <c r="V10" s="14"/>
-      <c r="W10" s="14"/>
-      <c r="X10" s="14"/>
-      <c r="Y10" s="14"/>
-      <c r="Z10" s="14"/>
+      <c r="T10" s="99"/>
+      <c r="U10" s="99"/>
+      <c r="V10" s="99"/>
+      <c r="W10" s="99"/>
+      <c r="X10" s="99"/>
+      <c r="Y10" s="99"/>
+      <c r="Z10" s="99"/>
     </row>
     <row r="11" ht="13.2" spans="1:26">
       <c r="A11" s="21"/>
@@ -13126,13 +13348,13 @@
       <c r="Q11" s="24"/>
       <c r="R11" s="24"/>
       <c r="S11" s="24"/>
-      <c r="T11" s="14"/>
-      <c r="U11" s="14"/>
-      <c r="V11" s="14"/>
-      <c r="W11" s="14"/>
-      <c r="X11" s="14"/>
-      <c r="Y11" s="14"/>
-      <c r="Z11" s="14"/>
+      <c r="T11" s="99"/>
+      <c r="U11" s="99"/>
+      <c r="V11" s="99"/>
+      <c r="W11" s="99"/>
+      <c r="X11" s="99"/>
+      <c r="Y11" s="99"/>
+      <c r="Z11" s="99"/>
     </row>
     <row r="12" ht="13.2" spans="1:26">
       <c r="A12" s="21"/>
@@ -13154,13 +13376,13 @@
       <c r="Q12" s="24"/>
       <c r="R12" s="24"/>
       <c r="S12" s="24"/>
-      <c r="T12" s="14"/>
-      <c r="U12" s="14"/>
-      <c r="V12" s="14"/>
-      <c r="W12" s="14"/>
-      <c r="X12" s="14"/>
-      <c r="Y12" s="14"/>
-      <c r="Z12" s="14"/>
+      <c r="T12" s="99"/>
+      <c r="U12" s="99"/>
+      <c r="V12" s="99"/>
+      <c r="W12" s="99"/>
+      <c r="X12" s="99"/>
+      <c r="Y12" s="99"/>
+      <c r="Z12" s="99"/>
     </row>
     <row r="13" ht="24.75" customHeight="1" spans="1:26">
       <c r="A13" s="21"/>
@@ -13182,13 +13404,13 @@
       <c r="Q13" s="24"/>
       <c r="R13" s="24"/>
       <c r="S13" s="24"/>
-      <c r="T13" s="14"/>
-      <c r="U13" s="14"/>
-      <c r="V13" s="14"/>
-      <c r="W13" s="14"/>
-      <c r="X13" s="14"/>
-      <c r="Y13" s="14"/>
-      <c r="Z13" s="14"/>
+      <c r="T13" s="99"/>
+      <c r="U13" s="99"/>
+      <c r="V13" s="99"/>
+      <c r="W13" s="99"/>
+      <c r="X13" s="99"/>
+      <c r="Y13" s="99"/>
+      <c r="Z13" s="99"/>
     </row>
     <row r="14" ht="13.2" spans="1:26">
       <c r="A14" s="21"/>
@@ -13210,13 +13432,13 @@
       <c r="Q14" s="24"/>
       <c r="R14" s="24"/>
       <c r="S14" s="24"/>
-      <c r="T14" s="14"/>
-      <c r="U14" s="14"/>
-      <c r="V14" s="14"/>
-      <c r="W14" s="14"/>
-      <c r="X14" s="14"/>
-      <c r="Y14" s="14"/>
-      <c r="Z14" s="14"/>
+      <c r="T14" s="99"/>
+      <c r="U14" s="99"/>
+      <c r="V14" s="99"/>
+      <c r="W14" s="99"/>
+      <c r="X14" s="99"/>
+      <c r="Y14" s="99"/>
+      <c r="Z14" s="99"/>
     </row>
     <row r="15" ht="13.2" spans="1:26">
       <c r="A15" s="21"/>
@@ -13238,13 +13460,13 @@
       <c r="Q15" s="24"/>
       <c r="R15" s="24"/>
       <c r="S15" s="24"/>
-      <c r="T15" s="14"/>
-      <c r="U15" s="14"/>
-      <c r="V15" s="14"/>
-      <c r="W15" s="14"/>
-      <c r="X15" s="14"/>
-      <c r="Y15" s="14"/>
-      <c r="Z15" s="14"/>
+      <c r="T15" s="99"/>
+      <c r="U15" s="99"/>
+      <c r="V15" s="99"/>
+      <c r="W15" s="99"/>
+      <c r="X15" s="99"/>
+      <c r="Y15" s="99"/>
+      <c r="Z15" s="99"/>
     </row>
     <row r="16" ht="13.95" spans="1:26">
       <c r="A16" s="25"/>
@@ -13266,13 +13488,13 @@
       <c r="Q16" s="23"/>
       <c r="R16" s="23"/>
       <c r="S16" s="23"/>
-      <c r="T16" s="14"/>
-      <c r="U16" s="14"/>
-      <c r="V16" s="14"/>
-      <c r="W16" s="14"/>
-      <c r="X16" s="14"/>
-      <c r="Y16" s="14"/>
-      <c r="Z16" s="14"/>
+      <c r="T16" s="99"/>
+      <c r="U16" s="99"/>
+      <c r="V16" s="99"/>
+      <c r="W16" s="99"/>
+      <c r="X16" s="99"/>
+      <c r="Y16" s="99"/>
+      <c r="Z16" s="99"/>
     </row>
     <row r="17" ht="13.95" spans="1:26">
       <c r="A17" s="15">
@@ -13296,13 +13518,13 @@
       <c r="Q17" s="19"/>
       <c r="R17" s="19"/>
       <c r="S17" s="27"/>
-      <c r="T17" s="28"/>
-      <c r="U17" s="28"/>
-      <c r="V17" s="28"/>
-      <c r="W17" s="28"/>
-      <c r="X17" s="28"/>
-      <c r="Y17" s="28"/>
-      <c r="Z17" s="28"/>
+      <c r="T17" s="100"/>
+      <c r="U17" s="100"/>
+      <c r="V17" s="100"/>
+      <c r="W17" s="100"/>
+      <c r="X17" s="100"/>
+      <c r="Y17" s="100"/>
+      <c r="Z17" s="100"/>
     </row>
     <row r="18" ht="13.2" spans="1:26">
       <c r="A18" s="21"/>

</xml_diff>

<commit_message>
Center workbook letterheads across each report table
</commit_message>
<xml_diff>
--- a/assets/report_templates/MSME_Report_Blank.xlsx
+++ b/assets/report_templates/MSME_Report_Blank.xlsx
@@ -1572,10 +1572,42 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="13906500" cy="1580300"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="PESO Vinzons letterhead"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>1085850</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="13906500" cy="1580300"/>
     <xdr:pic>

</xml_diff>

<commit_message>
Center letterheads on populated header columns and simplify download names
</commit_message>
<xml_diff>
--- a/assets/report_templates/MSME_Report_Blank.xlsx
+++ b/assets/report_templates/MSME_Report_Blank.xlsx
@@ -1572,8 +1572,8 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>642938</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
@@ -1604,8 +1604,8 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>1085850</xdr:colOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>280988</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>

</xml_diff>